<commit_message>
fix(full-estimate): align review workbook visuals
</commit_message>
<xml_diff>
--- a/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
+++ b/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
@@ -16,10 +16,10 @@
     <sheet name="06_Raw contracts" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_Конструктор сметы'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Проверка проекта'!$A$4:$N$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_Конструктор сметы'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Проверка проекта'!$A$4:$M$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Цены себестоимости'!$A$1:$P$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Детали объемов'!$A$1:$R$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Детали объемов'!$A$1:$P$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_Инструкция'!$A$1:$B$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Контракты'!$A$1:$I$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_Raw contracts'!$A$1:$C$15</definedName>
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,10 +51,16 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -68,7 +74,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="00666666"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -121,10 +132,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -134,6 +145,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -501,18 +515,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="72" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -538,25 +549,10 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Строк проверки</t>
+          <t>Что сейчас проверяется</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Цены</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Детализации</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Строк сметы</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Комментарий</t>
         </is>
@@ -583,67 +579,197 @@
           <t>reference_ready</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Reference contract from existing earthworks review-to-calculator flow; no project-specific values.</t>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>проверка проектных данных, цен и деталей</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>строки проверки: 7; цены: 12; детали: 2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
+          <t>Фундаментная плита</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>foundation_slab</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>позже</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Гидроизоляция</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Production contract: no old project values, fixture totals, or Excel-match overrides.</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>проверка проектных данных, цен и деталей</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>строки проверки: 2; цены: 6; детали: 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>load_bearing_walls_lintels</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>позже</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Перекрытие 1 этажа</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>floor_slab_1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>позже</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Перекрытие 2 этажа</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>floor_slab_2</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>позже</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Кровля</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>flat_roof</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>позже</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Schiedel / вентканалы</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>schiedel_vent_channels</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>позже</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
+  <autoFilter ref="A1:F9"/>
   <dataValidations count="1">
-    <dataValidation sqref="C2:C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C2:C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"да,нет"</formula1>
     </dataValidation>
   </dataValidations>
@@ -657,29 +783,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
-    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="64" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
     <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col hidden="1" width="20" customWidth="1" min="11" max="11"/>
-    <col hidden="1" width="28" customWidth="1" min="12" max="12"/>
-    <col hidden="1" width="18" customWidth="1" min="13" max="13"/>
-    <col hidden="1" width="24" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="20" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="28" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="18" customWidth="1" min="12" max="12"/>
+    <col hidden="1" width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Review workbook: проектные входы из section contracts</t>
+          <t>Разбор проекта:
+земляные работы + гидроизоляция</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr"/>
@@ -694,21 +820,28 @@
       <c r="K1" s="2" t="inlineStr"/>
       <c r="L1" s="2" t="inlineStr"/>
       <c r="M1" s="2" t="inlineStr"/>
-      <c r="N1" s="2" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Проверочный лист</t>
+          <t>Найдено уверенно: 0</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Значения здесь должны приходить из parser/chat JSON или ручной правки.</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+          <t>Проверьте: 9</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Не найдено: 0</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ручной ввод: 0</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
@@ -716,9 +849,8 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -734,75 +866,69 @@
       <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Раздел</t>
+          <t>Что проверяем</t>
         </is>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Что проверяем</t>
+          <t>Найдено в проекте</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>Найдено в проекте</t>
+          <t>Ед.</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>Ед.</t>
+          <t>Статус</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Статус</t>
+          <t>Что нужно сделать</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>Что нужно сделать</t>
+          <t>Источник</t>
         </is>
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Источник</t>
+          <t>Фрагмент проекта</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Фрагмент проекта</t>
+          <t>Исправить / ввести значение</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
         <is>
-          <t>Исправить / ввести значение</t>
+          <t>Комментарий Елены</t>
         </is>
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t>Комментарий Елены</t>
+          <t>section_code</t>
         </is>
       </c>
       <c r="K4" s="1" t="inlineStr">
         <is>
-          <t>section_code</t>
+          <t>technical_key</t>
         </is>
       </c>
       <c r="L4" s="1" t="inlineStr">
         <is>
-          <t>technical_key</t>
+          <t>source_class</t>
         </is>
       </c>
       <c r="M4" s="1" t="inlineStr">
-        <is>
-          <t>source_class</t>
-        </is>
-      </c>
-      <c r="N4" s="1" t="inlineStr">
         <is>
           <t>target_code</t>
         </is>
@@ -814,11 +940,7 @@
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>earthworks</t>
-        </is>
-      </c>
+      <c r="B5" s="4" t="inlineStr"/>
       <c r="C5" s="4" t="inlineStr"/>
       <c r="D5" s="4" t="inlineStr"/>
       <c r="E5" s="4" t="inlineStr"/>
@@ -830,55 +952,49 @@
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr"/>
       <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
           <t>Площадь котлована</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
           <t>Проверьте площадь котлована из проекта.</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="inlineStr"/>
-      <c r="J6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>pit_area_m2</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>pit_area_m2</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>pit_area_m2</t>
         </is>
@@ -887,50 +1003,45 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
           <t>Глубина котлована</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>м</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
           <t>Проверьте глубину котлована.</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>pit_excavation_depth_m</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>pit_excavation_depth_m</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
         <is>
           <t>pit_excavation_depth_m</t>
         </is>
@@ -939,50 +1050,45 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
           <t>Объем песка под основание</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>м3</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
           <t>Проверьте объем песка из спецификации.</t>
         </is>
       </c>
+      <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>sand_base_volume_m3</t>
         </is>
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>sand_base_volume_m3</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N8" s="5" t="inlineStr">
         <is>
           <t>sand_base_volume_m3</t>
         </is>
@@ -991,50 +1097,45 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
           <t>Объем траншей</t>
         </is>
       </c>
-      <c r="C9" s="5" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>м3</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
           <t>Проверьте общий объем траншей.</t>
         </is>
       </c>
+      <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>trench_volume_m3</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>trench_volume_m3</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N9" s="5" t="inlineStr">
         <is>
           <t>trench_volume_m3</t>
         </is>
@@ -1043,50 +1144,45 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
           <t>Площадь геотекстиля</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
           <t>Проверьте площадь материала геотекстиля.</t>
         </is>
       </c>
+      <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr"/>
       <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K10" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>geotextile_area_m2</t>
         </is>
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>geotextile_area_m2</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N10" s="5" t="inlineStr">
         <is>
           <t>geotextile_area_m2</t>
         </is>
@@ -1095,50 +1191,45 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
           <t>Площадь укладки геотекстиля</t>
         </is>
       </c>
-      <c r="C11" s="5" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
           <t>Проверьте площадь укладки геотекстиля.</t>
         </is>
       </c>
+      <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>geotextile_laying_area_m2</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>geotextile_laying_area_m2</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
         <is>
           <t>geotextile_laying_area_m2</t>
         </is>
@@ -1147,50 +1238,45 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
           <t>Длина коммуникаций</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>м</t>
+        </is>
+      </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>м</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
           <t>Проверьте длину коммуникаций и состав труб на листе деталей.</t>
         </is>
       </c>
+      <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
-      <c r="J12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>communications_length_m</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>communications_length_m</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M12" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
         <is>
           <t>communications_length_m</t>
         </is>
@@ -1202,11 +1288,7 @@
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>waterproofing</t>
-        </is>
-      </c>
+      <c r="B13" s="4" t="inlineStr"/>
       <c r="C13" s="4" t="inlineStr"/>
       <c r="D13" s="4" t="inlineStr"/>
       <c r="E13" s="4" t="inlineStr"/>
@@ -1218,55 +1300,49 @@
       <c r="K13" s="4" t="inlineStr"/>
       <c r="L13" s="4" t="inlineStr"/>
       <c r="M13" s="4" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
           <t>Площадь гидроизоляции фундаментной плиты</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n"/>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
           <t>Проверьте площадь гидроизоляции из спецификации.</t>
         </is>
       </c>
+      <c r="F14" s="5" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr"/>
       <c r="H14" s="5" t="inlineStr"/>
       <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>waterproofing</t>
+        </is>
+      </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>waterproofing_area_m2</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>waterproofing_area_m2</t>
+          <t>AUTO_PROJECT</t>
         </is>
       </c>
       <c r="M14" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
         <is>
           <t>waterproofing_area_m2</t>
         </is>
@@ -1275,57 +1351,52 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
           <t>ЭППС 100 мм по торцу фундаментной плиты, объем</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n"/>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>м3</t>
+          <t>Проверьте</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Ожидает извлечения</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
           <t>Проверьте объем ЭППС 100 мм по торцу фундаментной плиты.</t>
         </is>
       </c>
+      <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>waterproofing</t>
+        </is>
+      </c>
       <c r="K15" s="5" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>eps100_wall_volume_m3</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
+          <t>AUTO_PROJECT</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
           <t>eps100_wall_volume_m3</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
-        <is>
-          <t>AUTO_PROJECT</t>
-        </is>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>eps100_wall_volume_m3</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N15"/>
+  <autoFilter ref="A4:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1466,748 +1537,748 @@
       <c r="P2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Разбивка осей</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>смена</t>
         </is>
       </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="M3" s="6" t="inlineStr">
         <is>
           <t>axis_marking_work_unit_price</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>axis_marking_shift</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O3" s="6" t="inlineStr">
         <is>
           <t>axis_marking_work_unit_price</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr"/>
+      <c r="P3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Экскаватор JCB, материал/аренда</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>смена</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>excavator_material_unit_price</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>excavator_jcb_shift</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>excavator_material_unit_price</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr"/>
+      <c r="P4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Экскаватор JCB, работа</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>смена</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>excavator_work_unit_price</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>excavator_jcb_shift</t>
         </is>
       </c>
-      <c r="O5" s="5" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>excavator_work_unit_price</t>
         </is>
       </c>
-      <c r="P5" s="5" t="inlineStr"/>
+      <c r="P5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Доработка грунта вручную</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>м3</t>
         </is>
       </c>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="inlineStr"/>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="inlineStr"/>
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>manual_excavation_work_unit_price</t>
         </is>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>manual_excavation_m3</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>manual_excavation_work_unit_price</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr"/>
+      <c r="P6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Укладка геотекстиля</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>м2</t>
         </is>
       </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J7" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L7" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="M7" s="6" t="inlineStr">
         <is>
           <t>geotextile_laying_work_unit_price</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>geotextile_laying_m2</t>
         </is>
       </c>
-      <c r="O7" s="5" t="inlineStr">
+      <c r="O7" s="6" t="inlineStr">
         <is>
           <t>geotextile_laying_work_unit_price</t>
         </is>
       </c>
-      <c r="P7" s="5" t="inlineStr"/>
+      <c r="P7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Геотекстиль</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>м2</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="inlineStr"/>
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="L8" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
+      <c r="M8" s="6" t="inlineStr">
         <is>
           <t>geotextile_material_unit_price</t>
         </is>
       </c>
-      <c r="N8" s="5" t="inlineStr">
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>geotextile_dornit_300_m2</t>
         </is>
       </c>
-      <c r="O8" s="5" t="inlineStr">
+      <c r="O8" s="6" t="inlineStr">
         <is>
           <t>geotextile_material_unit_price</t>
         </is>
       </c>
-      <c r="P8" s="5" t="inlineStr"/>
+      <c r="P8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Засыпка песком</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>м3</t>
         </is>
       </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>sand_filling_work_unit_price</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>sand_filling_work_m3</t>
         </is>
       </c>
-      <c r="O9" s="5" t="inlineStr">
+      <c r="O9" s="6" t="inlineStr">
         <is>
           <t>sand_filling_work_unit_price</t>
         </is>
       </c>
-      <c r="P9" s="5" t="inlineStr"/>
+      <c r="P9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Песок</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>м3</t>
         </is>
       </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>sand_material_unit_price</t>
         </is>
       </c>
-      <c r="N10" s="5" t="inlineStr">
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>sand_m3</t>
         </is>
       </c>
-      <c r="O10" s="5" t="inlineStr">
+      <c r="O10" s="6" t="inlineStr">
         <is>
           <t>sand_material_unit_price</t>
         </is>
       </c>
-      <c r="P10" s="5" t="inlineStr"/>
+      <c r="P10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Перемещение песка вручную</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>м3</t>
         </is>
       </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="inlineStr"/>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>sand_manual_moving_work_unit_price</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>sand_manual_moving_m3</t>
         </is>
       </c>
-      <c r="O11" s="5" t="inlineStr">
+      <c r="O11" s="6" t="inlineStr">
         <is>
           <t>sand_manual_moving_work_unit_price</t>
         </is>
       </c>
-      <c r="P11" s="5" t="inlineStr"/>
+      <c r="P11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Монтаж коммуникаций</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>м</t>
         </is>
       </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="inlineStr"/>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="inlineStr"/>
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>communications_work_unit_price</t>
         </is>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>communications_installation_m</t>
         </is>
       </c>
-      <c r="O12" s="5" t="inlineStr">
+      <c r="O12" s="6" t="inlineStr">
         <is>
           <t>communications_work_unit_price</t>
         </is>
       </c>
-      <c r="P12" s="5" t="inlineStr"/>
+      <c r="P12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Материалы коммуникаций</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>м</t>
         </is>
       </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="inlineStr"/>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>communications_material_unit_price</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>communications_material_m</t>
         </is>
       </c>
-      <c r="O13" s="5" t="inlineStr">
+      <c r="O13" s="6" t="inlineStr">
         <is>
           <t>communications_material_unit_price</t>
         </is>
       </c>
-      <c r="P13" s="5" t="inlineStr"/>
+      <c r="P13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Расходные материалы</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Фиксированная строка</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>комплект</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>consumables_amount</t>
         </is>
       </c>
-      <c r="N14" s="5" t="inlineStr">
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>earthworks_consumables_fixed</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr">
+      <c r="O14" s="6" t="inlineStr">
         <is>
           <t>consumables_amount</t>
         </is>
       </c>
-      <c r="P14" s="5" t="inlineStr"/>
+      <c r="P14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -2236,376 +2307,376 @@
       <c r="P15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция битумной мастикой, работа</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>м2</t>
         </is>
       </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="inlineStr"/>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="inlineStr"/>
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>waterproofing_work_unit_price</t>
         </is>
       </c>
-      <c r="N16" s="5" t="inlineStr">
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>bitumen_waterproofing_work_m2</t>
         </is>
       </c>
-      <c r="O16" s="5" t="inlineStr">
+      <c r="O16" s="6" t="inlineStr">
         <is>
           <t>waterproofing_work_unit_price</t>
         </is>
       </c>
-      <c r="P16" s="5" t="inlineStr"/>
+      <c r="P16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Праймер битумный AquaMast, 18 л</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="inlineStr"/>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
         <is>
           <t>primer_unit_price</t>
         </is>
       </c>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>bitumen_primer_aquamast_18l_item</t>
         </is>
       </c>
-      <c r="O17" s="5" t="inlineStr">
+      <c r="O17" s="6" t="inlineStr">
         <is>
           <t>primer_unit_price</t>
         </is>
       </c>
-      <c r="P17" s="5" t="inlineStr"/>
+      <c r="P17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Мастика гидроизоляционная AquaMast, 18 кг</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>шт</t>
         </is>
       </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="inlineStr"/>
-      <c r="I18" s="5" t="inlineStr">
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr">
+      <c r="L18" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="M18" s="5" t="inlineStr">
+      <c r="M18" s="6" t="inlineStr">
         <is>
           <t>mastic_unit_price</t>
         </is>
       </c>
-      <c r="N18" s="5" t="inlineStr">
+      <c r="N18" s="6" t="inlineStr">
         <is>
           <t>bitumen_mastic_aquamast_18kg_item</t>
         </is>
       </c>
-      <c r="O18" s="5" t="inlineStr">
+      <c r="O18" s="6" t="inlineStr">
         <is>
           <t>mastic_unit_price</t>
         </is>
       </c>
-      <c r="P18" s="5" t="inlineStr"/>
+      <c r="P18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Утепление торца плиты ЭППС 100 мм, работа</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Работа</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>м2</t>
         </is>
       </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="inlineStr"/>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="L19" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="M19" s="6" t="inlineStr">
         <is>
           <t>eps100_wall_insulation_work_unit_price</t>
         </is>
       </c>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>eps_wall_insulation_work_m2</t>
         </is>
       </c>
-      <c r="O19" s="5" t="inlineStr">
+      <c r="O19" s="6" t="inlineStr">
         <is>
           <t>eps100_wall_insulation_work_unit_price</t>
         </is>
       </c>
-      <c r="P19" s="5" t="inlineStr"/>
+      <c r="P19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Пеноплэкс ГЕО 100 мм</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D20" s="6" t="inlineStr">
         <is>
           <t>м3</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="inlineStr"/>
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J20" s="5" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
         <is>
           <t>eps100_unit_price</t>
         </is>
       </c>
-      <c r="N20" s="5" t="inlineStr">
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>eps_geo_100_m3</t>
         </is>
       </c>
-      <c r="O20" s="5" t="inlineStr">
+      <c r="O20" s="6" t="inlineStr">
         <is>
           <t>eps100_unit_price</t>
         </is>
       </c>
-      <c r="P20" s="5" t="inlineStr"/>
+      <c r="P20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Клей-пена для ЭППС</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>баллон</t>
         </is>
       </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="inlineStr"/>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr">
         <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="L21" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr">
         <is>
           <t>glue_foam_unit_price</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>eps_foam_glue_can</t>
         </is>
       </c>
-      <c r="O21" s="5" t="inlineStr">
+      <c r="O21" s="6" t="inlineStr">
         <is>
           <t>glue_foam_unit_price</t>
         </is>
       </c>
-      <c r="P21" s="5" t="inlineStr"/>
+      <c r="P21" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:P21"/>
@@ -2619,116 +2690,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="34" customWidth="1" min="14" max="14"/>
-    <col width="54" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col hidden="1" width="20" customWidth="1" min="17" max="17"/>
-    <col hidden="1" width="26" customWidth="1" min="18" max="18"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="78" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="20" customWidth="1" min="15" max="15"/>
+    <col hidden="1" width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Раздел</t>
+          <t>Тип</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Таблица</t>
+          <t>Наименование</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Тип</t>
+          <t>Длина, м</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Наименование</t>
+          <t>Глубина, м</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Длина, м</t>
+          <t>Ширина, м</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Глубина, м</t>
+          <t>Объем, м3</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Ширина, м</t>
+          <t>Диаметр, мм</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Объем, м3</t>
+          <t>Длина одной, м</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Диаметр, мм</t>
+          <t>Количество</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Длина одной, м</t>
+          <t>Итоговая длина, м</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Количество</t>
+          <t>Включено</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Итоговая длина, м</t>
+          <t>Источник</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Включено</t>
+          <t>Фрагмент проекта</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Источник</t>
+          <t>Комментарий Елены</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Фрагмент проекта</t>
+          <t>section_code</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Комментарий Елены</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>section_code</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>detail_table_key</t>
         </is>
@@ -2740,11 +2799,7 @@
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>earthworks</t>
-        </is>
-      </c>
+      <c r="B2" s="4" t="inlineStr"/>
       <c r="C2" s="4" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr"/>
       <c r="E2" s="4" t="inlineStr"/>
@@ -2759,135 +2814,113 @@
       <c r="N2" s="4" t="inlineStr"/>
       <c r="O2" s="4" t="inlineStr"/>
       <c r="P2" s="4" t="inlineStr"/>
-      <c r="Q2" s="4" t="inlineStr"/>
-      <c r="R2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Маршруты траншей</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Шаблон строк</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Длина, м</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Глубина, м</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Ширина, м</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Объем, м3</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="6" t="inlineStr"/>
-      <c r="K3" s="6" t="inlineStr"/>
-      <c r="L3" s="6" t="inlineStr"/>
-      <c r="M3" s="6" t="inlineStr"/>
-      <c r="N3" s="6" t="inlineStr"/>
-      <c r="O3" s="6" t="inlineStr"/>
-      <c r="P3" s="6" t="inlineStr"/>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr"/>
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
+      <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="7" t="inlineStr"/>
+      <c r="O3" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="R3" s="6" t="inlineStr">
+      <c r="P3" s="7" t="inlineStr">
         <is>
           <t>trench_routes</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Трубы коммуникаций</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Шаблон строк</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Наименование</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr"/>
-      <c r="F4" s="6" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr"/>
-      <c r="H4" s="6" t="inlineStr"/>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Диаметр, мм</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Длина одной, м</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
         <is>
           <t>Количество, шт</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Итоговая длина, м</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="K4" s="7" t="inlineStr">
         <is>
           <t>Включено</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr"/>
-      <c r="O4" s="6" t="inlineStr"/>
-      <c r="P4" s="6" t="inlineStr"/>
-      <c r="Q4" s="6" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr"/>
+      <c r="M4" s="7" t="inlineStr"/>
+      <c r="N4" s="7" t="inlineStr"/>
+      <c r="O4" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="R4" s="6" t="inlineStr">
+      <c r="P4" s="7" t="inlineStr">
         <is>
           <t>communications_pipe_items</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R4"/>
+  <autoFilter ref="A1:P4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3063,70 +3096,70 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="D2" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="E2" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="7" t="n">
+      <c r="F2" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="G2" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="7" t="n">
+      <c r="H2" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>{"calculator": "experiments/earthworks_calculator/earthworks_calculator.py", "calculator_readme": "experiments/earthworks_calculator/README.md", "existing_cases": [], "related_docs": ["experiments/full_estimate_review_pipeline/reports/step_01_earthworks_reference.md", "docs/report_earthworks_parser_google_stage1.md", "docs/report_earthworks_review_to_calculator.md"], "extraction_targets": ["experiments/chat_extraction_poc/data/calculator_targets_compact.json", "experiments/chat_extraction_poc/data/target_aliases_ru.yaml"]}</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="C3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="7" t="n">
+      <c r="D3" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="E3" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="7" t="n">
+      <c r="F3" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="G3" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="H3" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
         <is>
           <t>{"calculator": "experiments/waterproofing_calculator/waterproofing_calculator.py", "calculator_readme": "experiments/waterproofing_calculator/README.md", "existing_cases": ["experiments/waterproofing_calculator/cases/test_waterproofing_spec_area"], "related_docs": ["experiments/full_estimate_review_pipeline/reports/step_03_all_sections_quantity_matrix.md", "experiments/full_estimate_review_pipeline/reports/step_03b_production_contamination_audit.md", "docs/elena_parameter_review_pack_audit.md", "docs/report_paid_waterproofing_calculator_changes.md", "docs/report_waterproofing_calculator.md"], "extraction_targets": ["experiments/chat_extraction_poc/data/calculator_targets_compact.json", "experiments/chat_extraction_poc/data/target_aliases_ru.yaml"]}</t>
         </is>
@@ -3170,17 +3203,17 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>{
   "code": "earthworks",
@@ -3193,17 +3226,17 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -3453,17 +3486,17 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -3627,17 +3660,17 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -3774,17 +3807,17 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -3913,17 +3946,17 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -3967,17 +4000,17 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -4318,17 +4351,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>{
   "code": "waterproofing",
@@ -4341,17 +4374,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -4431,17 +4464,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -4527,34 +4560,34 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -4716,17 +4749,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>[
   {
@@ -4880,17 +4913,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>[
   {

</xml_diff>

<commit_message>
fix(full-estimate): refine review workbook sheets
</commit_message>
<xml_diff>
--- a/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
+++ b/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
@@ -12,18 +12,10 @@
     <sheet name="02_Цены себестоимости" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="03_Детали объемов" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="04_Инструкция" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="05_Контракты" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="06_Raw contracts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="05_Кандидаты parser" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_Сырые данные parser" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_Конструктор сметы'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_Проверка проекта'!$A$4:$M$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Цены себестоимости'!$A$1:$P$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Детали объемов'!$A$1:$P$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_Инструкция'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Контракты'!$A$1:$I$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_Raw contracts'!$A$1:$C$15</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -767,7 +759,6 @@
       <c r="F9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F9"/>
   <dataValidations count="1">
     <dataValidation sqref="C2:C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"да,нет"</formula1>
@@ -1396,7 +1387,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1407,1279 +1397,1130 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="58" customWidth="1" min="11" max="11"/>
-    <col hidden="1" width="20" customWidth="1" min="12" max="12"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="66" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="20" customWidth="1" min="11" max="11"/>
+    <col hidden="1" width="30" customWidth="1" min="12" max="12"/>
     <col hidden="1" width="30" customWidth="1" min="13" max="13"/>
     <col hidden="1" width="30" customWidth="1" min="14" max="14"/>
-    <col hidden="1" width="30" customWidth="1" min="15" max="15"/>
-    <col hidden="1" width="22" customWidth="1" min="16" max="16"/>
+    <col hidden="1" width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Раздел</t>
+          <t>Строка сметы</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Строка сметы</t>
+          <t>Что это за цена</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Что это за цена</t>
+          <t>Ед.</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Ед.</t>
+          <t>Цена из прайса</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Цена из прайса</t>
+          <t>Цена fallback</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Цена fallback</t>
+          <t>Цена для расчета</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Цена для расчета</t>
+          <t>Исправить цену</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Исправить цену</t>
+          <t>Источник цены</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Источник цены</t>
+          <t>Нужно внимание</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Нужно внимание</t>
+          <t>Комментарий</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Комментарий</t>
+          <t>section_code</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>section_code</t>
+          <t>calc_price_key</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>calc_price_key</t>
+          <t>price_registry_code</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>price_registry_code</t>
+          <t>fallback_key</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>fallback_key</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
           <t>selected_price_source</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Земляные работы</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Разбивка осей</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Работа</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="6" t="inlineStr"/>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>Заполнить цену из price registry/fallback/review.</t>
+        </is>
+      </c>
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr"/>
-      <c r="F2" s="4" t="inlineStr"/>
-      <c r="G2" s="4" t="inlineStr"/>
-      <c r="H2" s="4" t="inlineStr"/>
-      <c r="I2" s="4" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr"/>
-      <c r="K2" s="4" t="inlineStr"/>
-      <c r="L2" s="4" t="inlineStr"/>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr"/>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>axis_marking_work_unit_price</t>
+        </is>
+      </c>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>axis_marking_shift</t>
+        </is>
+      </c>
+      <c r="N2" s="6" t="inlineStr">
+        <is>
+          <t>axis_marking_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Экскаватор JCB, материал/аренда</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Разбивка осей</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
           <t>смена</t>
         </is>
       </c>
+      <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
       <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr"/>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>excavator_material_unit_price</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>axis_marking_work_unit_price</t>
+          <t>excavator_jcb_shift</t>
         </is>
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>axis_marking_shift</t>
-        </is>
-      </c>
-      <c r="O3" s="6" t="inlineStr">
-        <is>
-          <t>axis_marking_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P3" s="6" t="inlineStr"/>
+          <t>excavator_material_unit_price</t>
+        </is>
+      </c>
+      <c r="O3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Экскаватор JCB, работа</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Экскаватор JCB, материал/аренда</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
           <t>смена</t>
         </is>
       </c>
+      <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
       <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>excavator_work_unit_price</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
         <is>
-          <t>excavator_material_unit_price</t>
+          <t>excavator_jcb_shift</t>
         </is>
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>excavator_jcb_shift</t>
-        </is>
-      </c>
-      <c r="O4" s="6" t="inlineStr">
-        <is>
-          <t>excavator_material_unit_price</t>
-        </is>
-      </c>
-      <c r="P4" s="6" t="inlineStr"/>
+          <t>excavator_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Доработка грунта вручную</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Экскаватор JCB, работа</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>смена</t>
-        </is>
-      </c>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr"/>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>manual_excavation_work_unit_price</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>excavator_work_unit_price</t>
+          <t>manual_excavation_m3</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>excavator_jcb_shift</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>excavator_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr"/>
+          <t>manual_excavation_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Укладка геотекстиля</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Доработка грунта вручную</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>м3</t>
-        </is>
-      </c>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
       <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="inlineStr"/>
+      <c r="G6" s="6" t="inlineStr"/>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>geotextile_laying_work_unit_price</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>manual_excavation_work_unit_price</t>
+          <t>geotextile_laying_m2</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>manual_excavation_m3</t>
-        </is>
-      </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>manual_excavation_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="inlineStr"/>
+          <t>geotextile_laying_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Геотекстиль</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Укладка геотекстиля</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
           <t>м2</t>
         </is>
       </c>
+      <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>geotextile_material_unit_price</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>geotextile_laying_work_unit_price</t>
+          <t>geotextile_dornit_300_m2</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>geotextile_laying_m2</t>
-        </is>
-      </c>
-      <c r="O7" s="6" t="inlineStr">
-        <is>
-          <t>geotextile_laying_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P7" s="6" t="inlineStr"/>
+          <t>geotextile_material_unit_price</t>
+        </is>
+      </c>
+      <c r="O7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Засыпка песком</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Геотекстиль</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>м2</t>
-        </is>
-      </c>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="inlineStr"/>
+      <c r="G8" s="6" t="inlineStr"/>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>sand_filling_work_unit_price</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>geotextile_material_unit_price</t>
+          <t>sand_filling_work_m3</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>geotextile_dornit_300_m2</t>
-        </is>
-      </c>
-      <c r="O8" s="6" t="inlineStr">
-        <is>
-          <t>geotextile_material_unit_price</t>
-        </is>
-      </c>
-      <c r="P8" s="6" t="inlineStr"/>
+          <t>sand_filling_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Песок</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Засыпка песком</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
           <t>м3</t>
         </is>
       </c>
+      <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>sand_material_unit_price</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>sand_filling_work_unit_price</t>
+          <t>sand_m3</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>sand_filling_work_m3</t>
-        </is>
-      </c>
-      <c r="O9" s="6" t="inlineStr">
-        <is>
-          <t>sand_filling_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P9" s="6" t="inlineStr"/>
+          <t>sand_material_unit_price</t>
+        </is>
+      </c>
+      <c r="O9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Перемещение песка вручную</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Песок</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
           <t>м3</t>
         </is>
       </c>
+      <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
       <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>sand_manual_moving_work_unit_price</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>sand_material_unit_price</t>
+          <t>sand_manual_moving_m3</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>sand_m3</t>
-        </is>
-      </c>
-      <c r="O10" s="6" t="inlineStr">
-        <is>
-          <t>sand_material_unit_price</t>
-        </is>
-      </c>
-      <c r="P10" s="6" t="inlineStr"/>
+          <t>sand_manual_moving_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Монтаж коммуникаций</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Перемещение песка вручную</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>м3</t>
-        </is>
-      </c>
+          <t>м</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
       <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>communications_work_unit_price</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>sand_manual_moving_work_unit_price</t>
+          <t>communications_installation_m</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>sand_manual_moving_m3</t>
-        </is>
-      </c>
-      <c r="O11" s="6" t="inlineStr">
-        <is>
-          <t>sand_manual_moving_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="inlineStr"/>
+          <t>communications_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Материалы коммуникаций</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Монтаж коммуникаций</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
           <t>м</t>
         </is>
       </c>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
       <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="inlineStr"/>
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>communications_material_unit_price</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>communications_work_unit_price</t>
+          <t>communications_material_m</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>communications_installation_m</t>
-        </is>
-      </c>
-      <c r="O12" s="6" t="inlineStr">
-        <is>
-          <t>communications_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P12" s="6" t="inlineStr"/>
+          <t>communications_material_unit_price</t>
+        </is>
+      </c>
+      <c r="O12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Расходные материалы</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Материалы коммуникаций</t>
+          <t>Фиксированная строка</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>м</t>
-        </is>
-      </c>
+          <t>комплект</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr"/>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>earthworks</t>
+          <t>consumables_amount</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>communications_material_unit_price</t>
+          <t>earthworks_consumables_fixed</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>communications_material_m</t>
-        </is>
-      </c>
-      <c r="O13" s="6" t="inlineStr">
-        <is>
-          <t>communications_material_unit_price</t>
-        </is>
-      </c>
-      <c r="P13" s="6" t="inlineStr"/>
+          <t>consumables_amount</t>
+        </is>
+      </c>
+      <c r="O13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Земляные работы</t>
+          <t>Гидроизоляция битумной мастикой, работа</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Расходные материалы</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Фиксированная строка</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>комплект</t>
-        </is>
-      </c>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Заполнить цену из price registry/fallback/review.</t>
+        </is>
+      </c>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>waterproofing</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>waterproofing_work_unit_price</t>
+        </is>
+      </c>
+      <c r="M14" s="6" t="inlineStr">
+        <is>
+          <t>bitumen_waterproofing_work_m2</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
+        <is>
+          <t>waterproofing_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Праймер битумный AquaMast, 18 л</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
           <t>price_registry_with_fallback</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>да</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
-        <is>
-          <t>earthworks</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="inlineStr">
-        <is>
-          <t>consumables_amount</t>
-        </is>
-      </c>
-      <c r="N14" s="6" t="inlineStr">
-        <is>
-          <t>earthworks_consumables_fixed</t>
-        </is>
-      </c>
-      <c r="O14" s="6" t="inlineStr">
-        <is>
-          <t>consumables_amount</t>
-        </is>
-      </c>
-      <c r="P14" s="6" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Гидроизоляция фундаментной плиты</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr"/>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr"/>
-      <c r="I15" s="4" t="inlineStr"/>
-      <c r="J15" s="4" t="inlineStr"/>
-      <c r="K15" s="4" t="inlineStr"/>
-      <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="4" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr"/>
-      <c r="O15" s="4" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr"/>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>primer_unit_price</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="inlineStr">
+        <is>
+          <t>bitumen_primer_aquamast_18l_item</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
+        <is>
+          <t>primer_unit_price</t>
+        </is>
+      </c>
+      <c r="O15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
+          <t>Мастика гидроизоляционная AquaMast, 18 кг</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Гидроизоляция битумной мастикой, работа</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>м2</t>
-        </is>
-      </c>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="inlineStr"/>
+      <c r="G16" s="6" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>waterproofing</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>mastic_unit_price</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>waterproofing_work_unit_price</t>
+          <t>bitumen_mastic_aquamast_18kg_item</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>bitumen_waterproofing_work_m2</t>
-        </is>
-      </c>
-      <c r="O16" s="6" t="inlineStr">
-        <is>
-          <t>waterproofing_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P16" s="6" t="inlineStr"/>
+          <t>mastic_unit_price</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
+          <t>Утепление торца плиты ЭППС 100 мм, работа</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Праймер битумный AquaMast, 18 л</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>waterproofing</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>eps100_wall_insulation_work_unit_price</t>
         </is>
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>primer_unit_price</t>
+          <t>eps_wall_insulation_work_m2</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>bitumen_primer_aquamast_18l_item</t>
-        </is>
-      </c>
-      <c r="O17" s="6" t="inlineStr">
-        <is>
-          <t>primer_unit_price</t>
-        </is>
-      </c>
-      <c r="P17" s="6" t="inlineStr"/>
+          <t>eps100_wall_insulation_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
+          <t>Пеноплэкс ГЕО 100 мм</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Мастика гидроизоляционная AquaMast, 18 кг</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J18" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>waterproofing</t>
         </is>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>eps100_unit_price</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>mastic_unit_price</t>
+          <t>eps_geo_100_m3</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>bitumen_mastic_aquamast_18kg_item</t>
-        </is>
-      </c>
-      <c r="O18" s="6" t="inlineStr">
-        <is>
-          <t>mastic_unit_price</t>
-        </is>
-      </c>
-      <c r="P18" s="6" t="inlineStr"/>
+          <t>eps100_unit_price</t>
+        </is>
+      </c>
+      <c r="O18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Гидроизоляция фундаментной плиты</t>
+          <t>Клей-пена для ЭППС</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Утепление торца плиты ЭППС 100 мм, работа</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>м2</t>
-        </is>
-      </c>
+          <t>баллон</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>price_registry_with_fallback</t>
+          <t>да</t>
         </is>
       </c>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>да</t>
+          <t>Заполнить цену из price registry/fallback/review.</t>
         </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
+          <t>waterproofing</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>glue_foam_unit_price</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>eps100_wall_insulation_work_unit_price</t>
+          <t>eps_foam_glue_can</t>
         </is>
       </c>
       <c r="N19" s="6" t="inlineStr">
         <is>
-          <t>eps_wall_insulation_work_m2</t>
-        </is>
-      </c>
-      <c r="O19" s="6" t="inlineStr">
-        <is>
-          <t>eps100_wall_insulation_work_unit_price</t>
-        </is>
-      </c>
-      <c r="P19" s="6" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Гидроизоляция фундаментной плиты</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>Пеноплэкс ГЕО 100 мм</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>м3</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="inlineStr"/>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>price_registry_with_fallback</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
-        </is>
-      </c>
-      <c r="L20" s="6" t="inlineStr">
-        <is>
-          <t>waterproofing</t>
-        </is>
-      </c>
-      <c r="M20" s="6" t="inlineStr">
-        <is>
-          <t>eps100_unit_price</t>
-        </is>
-      </c>
-      <c r="N20" s="6" t="inlineStr">
-        <is>
-          <t>eps_geo_100_m3</t>
-        </is>
-      </c>
-      <c r="O20" s="6" t="inlineStr">
-        <is>
-          <t>eps100_unit_price</t>
-        </is>
-      </c>
-      <c r="P20" s="6" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Гидроизоляция фундаментной плиты</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>Клей-пена для ЭППС</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>баллон</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="inlineStr"/>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>price_registry_with_fallback</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
-        </is>
-      </c>
-      <c r="L21" s="6" t="inlineStr">
-        <is>
-          <t>waterproofing</t>
-        </is>
-      </c>
-      <c r="M21" s="6" t="inlineStr">
-        <is>
           <t>glue_foam_unit_price</t>
         </is>
       </c>
-      <c r="N21" s="6" t="inlineStr">
-        <is>
-          <t>eps_foam_glue_can</t>
-        </is>
-      </c>
-      <c r="O21" s="6" t="inlineStr">
-        <is>
-          <t>glue_foam_unit_price</t>
-        </is>
-      </c>
-      <c r="P21" s="6" t="inlineStr"/>
+      <c r="O19" s="6" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2920,7 +2761,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2934,7 +2774,7 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="120" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2951,10 +2791,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>00</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -2963,10 +2801,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
@@ -2975,10 +2811,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -2987,10 +2821,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -2999,10 +2831,8 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>05</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -3011,19 +2841,16 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Raw contracts нужен разработчику для диагностики структуры.</t>
+          <t>Сырые данные parser нужны разработчику для диагностики структуры.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3166,7 +2993,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5245,7 +5071,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refine full estimate review workbook templates
</commit_message>
<xml_diff>
--- a/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
+++ b/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -138,6 +138,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1397,7 +1403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1495,71 +1501,35 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Разбивка осей</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Работа</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>смена</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="inlineStr"/>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>price_registry_with_fallback</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>earthworks</t>
-        </is>
-      </c>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>axis_marking_work_unit_price</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>axis_marking_shift</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>axis_marking_work_unit_price</t>
-        </is>
-      </c>
-      <c r="O2" s="6" t="inlineStr"/>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr"/>
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr"/>
+      <c r="E2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr"/>
+      <c r="H2" s="4" t="inlineStr"/>
+      <c r="I2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr"/>
+      <c r="K2" s="4" t="inlineStr"/>
+      <c r="L2" s="4" t="inlineStr"/>
+      <c r="M2" s="4" t="inlineStr"/>
+      <c r="N2" s="4" t="inlineStr"/>
+      <c r="O2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Экскаватор JCB, материал/аренда</t>
+          <t>Разбивка осей</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1593,17 +1563,17 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>excavator_material_unit_price</t>
+          <t>axis_marking_work_unit_price</t>
         </is>
       </c>
       <c r="M3" s="6" t="inlineStr">
         <is>
-          <t>excavator_jcb_shift</t>
+          <t>axis_marking_shift</t>
         </is>
       </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
-          <t>excavator_material_unit_price</t>
+          <t>axis_marking_work_unit_price</t>
         </is>
       </c>
       <c r="O3" s="6" t="inlineStr"/>
@@ -1611,12 +1581,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Экскаватор JCB, работа</t>
+          <t>Экскаватор JCB, материал/аренда</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -1650,7 +1620,7 @@
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>excavator_work_unit_price</t>
+          <t>excavator_material_unit_price</t>
         </is>
       </c>
       <c r="M4" s="6" t="inlineStr">
@@ -1660,7 +1630,7 @@
       </c>
       <c r="N4" s="6" t="inlineStr">
         <is>
-          <t>excavator_work_unit_price</t>
+          <t>excavator_material_unit_price</t>
         </is>
       </c>
       <c r="O4" s="6" t="inlineStr"/>
@@ -1668,7 +1638,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Доработка грунта вручную</t>
+          <t>Экскаватор JCB, работа</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1678,7 +1648,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>м3</t>
+          <t>смена</t>
         </is>
       </c>
       <c r="D5" s="6" t="n"/>
@@ -1707,17 +1677,17 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>manual_excavation_work_unit_price</t>
+          <t>excavator_work_unit_price</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>manual_excavation_m3</t>
+          <t>excavator_jcb_shift</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t>manual_excavation_work_unit_price</t>
+          <t>excavator_work_unit_price</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr"/>
@@ -1725,7 +1695,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Укладка геотекстиля</t>
+          <t>Доработка грунта вручную</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -1735,7 +1705,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>м3</t>
         </is>
       </c>
       <c r="D6" s="6" t="n"/>
@@ -1764,17 +1734,17 @@
       </c>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>geotextile_laying_work_unit_price</t>
+          <t>manual_excavation_work_unit_price</t>
         </is>
       </c>
       <c r="M6" s="6" t="inlineStr">
         <is>
-          <t>geotextile_laying_m2</t>
+          <t>manual_excavation_m3</t>
         </is>
       </c>
       <c r="N6" s="6" t="inlineStr">
         <is>
-          <t>geotextile_laying_work_unit_price</t>
+          <t>manual_excavation_work_unit_price</t>
         </is>
       </c>
       <c r="O6" s="6" t="inlineStr"/>
@@ -1782,12 +1752,12 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Геотекстиль</t>
+          <t>Укладка геотекстиля</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1821,17 +1791,17 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>geotextile_material_unit_price</t>
+          <t>geotextile_laying_work_unit_price</t>
         </is>
       </c>
       <c r="M7" s="6" t="inlineStr">
         <is>
-          <t>geotextile_dornit_300_m2</t>
+          <t>geotextile_laying_m2</t>
         </is>
       </c>
       <c r="N7" s="6" t="inlineStr">
         <is>
-          <t>geotextile_material_unit_price</t>
+          <t>geotextile_laying_work_unit_price</t>
         </is>
       </c>
       <c r="O7" s="6" t="inlineStr"/>
@@ -1839,17 +1809,17 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>Засыпка песком</t>
+          <t>Геотекстиль</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>м3</t>
+          <t>м2</t>
         </is>
       </c>
       <c r="D8" s="6" t="n"/>
@@ -1878,17 +1848,17 @@
       </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
-          <t>sand_filling_work_unit_price</t>
+          <t>geotextile_material_unit_price</t>
         </is>
       </c>
       <c r="M8" s="6" t="inlineStr">
         <is>
-          <t>sand_filling_work_m3</t>
+          <t>geotextile_dornit_300_m2</t>
         </is>
       </c>
       <c r="N8" s="6" t="inlineStr">
         <is>
-          <t>sand_filling_work_unit_price</t>
+          <t>geotextile_material_unit_price</t>
         </is>
       </c>
       <c r="O8" s="6" t="inlineStr"/>
@@ -1896,12 +1866,12 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Песок</t>
+          <t>Засыпка песком</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1935,17 +1905,17 @@
       </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
-          <t>sand_material_unit_price</t>
+          <t>sand_filling_work_unit_price</t>
         </is>
       </c>
       <c r="M9" s="6" t="inlineStr">
         <is>
-          <t>sand_m3</t>
+          <t>sand_filling_work_m3</t>
         </is>
       </c>
       <c r="N9" s="6" t="inlineStr">
         <is>
-          <t>sand_material_unit_price</t>
+          <t>sand_filling_work_unit_price</t>
         </is>
       </c>
       <c r="O9" s="6" t="inlineStr"/>
@@ -1953,12 +1923,12 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>Перемещение песка вручную</t>
+          <t>Песок</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1992,17 +1962,17 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>sand_manual_moving_work_unit_price</t>
+          <t>sand_material_unit_price</t>
         </is>
       </c>
       <c r="M10" s="6" t="inlineStr">
         <is>
-          <t>sand_manual_moving_m3</t>
+          <t>sand_m3</t>
         </is>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
-          <t>sand_manual_moving_work_unit_price</t>
+          <t>sand_material_unit_price</t>
         </is>
       </c>
       <c r="O10" s="6" t="inlineStr"/>
@@ -2010,7 +1980,7 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Монтаж коммуникаций</t>
+          <t>Перемещение песка вручную</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -2020,7 +1990,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>м</t>
+          <t>м3</t>
         </is>
       </c>
       <c r="D11" s="6" t="n"/>
@@ -2049,17 +2019,17 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>communications_work_unit_price</t>
+          <t>sand_manual_moving_work_unit_price</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>communications_installation_m</t>
+          <t>sand_manual_moving_m3</t>
         </is>
       </c>
       <c r="N11" s="6" t="inlineStr">
         <is>
-          <t>communications_work_unit_price</t>
+          <t>sand_manual_moving_work_unit_price</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr"/>
@@ -2067,12 +2037,12 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Материалы коммуникаций</t>
+          <t>Монтаж коммуникаций</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -2106,17 +2076,17 @@
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
-          <t>communications_material_unit_price</t>
+          <t>communications_work_unit_price</t>
         </is>
       </c>
       <c r="M12" s="6" t="inlineStr">
         <is>
-          <t>communications_material_m</t>
+          <t>communications_installation_m</t>
         </is>
       </c>
       <c r="N12" s="6" t="inlineStr">
         <is>
-          <t>communications_material_unit_price</t>
+          <t>communications_work_unit_price</t>
         </is>
       </c>
       <c r="O12" s="6" t="inlineStr"/>
@@ -2124,17 +2094,17 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Расходные материалы</t>
+          <t>Материалы коммуникаций</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Фиксированная строка</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>комплект</t>
+          <t>м</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
@@ -2163,17 +2133,17 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>consumables_amount</t>
+          <t>communications_material_unit_price</t>
         </is>
       </c>
       <c r="M13" s="6" t="inlineStr">
         <is>
-          <t>earthworks_consumables_fixed</t>
+          <t>communications_material_m</t>
         </is>
       </c>
       <c r="N13" s="6" t="inlineStr">
         <is>
-          <t>consumables_amount</t>
+          <t>communications_material_unit_price</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr"/>
@@ -2181,17 +2151,17 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Гидроизоляция битумной мастикой, работа</t>
+          <t>Расходные материалы</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
+          <t>Фиксированная строка</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>комплект</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
@@ -2215,97 +2185,61 @@
       </c>
       <c r="K14" s="6" t="inlineStr">
         <is>
-          <t>waterproofing</t>
+          <t>earthworks</t>
         </is>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
-          <t>waterproofing_work_unit_price</t>
+          <t>consumables_amount</t>
         </is>
       </c>
       <c r="M14" s="6" t="inlineStr">
         <is>
-          <t>bitumen_waterproofing_work_m2</t>
+          <t>earthworks_consumables_fixed</t>
         </is>
       </c>
       <c r="N14" s="6" t="inlineStr">
         <is>
-          <t>waterproofing_work_unit_price</t>
+          <t>consumables_amount</t>
         </is>
       </c>
       <c r="O14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Праймер битумный AquaMast, 18 л</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Материал</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>шт</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="inlineStr"/>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>price_registry_with_fallback</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>да</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>Заполнить цену из price registry/fallback/review.</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>waterproofing</t>
-        </is>
-      </c>
-      <c r="L15" s="6" t="inlineStr">
-        <is>
-          <t>primer_unit_price</t>
-        </is>
-      </c>
-      <c r="M15" s="6" t="inlineStr">
-        <is>
-          <t>bitumen_primer_aquamast_18l_item</t>
-        </is>
-      </c>
-      <c r="N15" s="6" t="inlineStr">
-        <is>
-          <t>primer_unit_price</t>
-        </is>
-      </c>
-      <c r="O15" s="6" t="inlineStr"/>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Гидроизоляция фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr"/>
+      <c r="K15" s="4" t="inlineStr"/>
+      <c r="L15" s="4" t="inlineStr"/>
+      <c r="M15" s="4" t="inlineStr"/>
+      <c r="N15" s="4" t="inlineStr"/>
+      <c r="O15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>Мастика гидроизоляционная AquaMast, 18 кг</t>
+          <t>Гидроизоляция битумной мастикой, работа</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>шт</t>
+          <t>м2</t>
         </is>
       </c>
       <c r="D16" s="6" t="n"/>
@@ -2334,17 +2268,17 @@
       </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
-          <t>mastic_unit_price</t>
+          <t>waterproofing_work_unit_price</t>
         </is>
       </c>
       <c r="M16" s="6" t="inlineStr">
         <is>
-          <t>bitumen_mastic_aquamast_18kg_item</t>
+          <t>bitumen_waterproofing_work_m2</t>
         </is>
       </c>
       <c r="N16" s="6" t="inlineStr">
         <is>
-          <t>mastic_unit_price</t>
+          <t>waterproofing_work_unit_price</t>
         </is>
       </c>
       <c r="O16" s="6" t="inlineStr"/>
@@ -2352,17 +2286,17 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Утепление торца плиты ЭППС 100 мм, работа</t>
+          <t>Праймер битумный AquaMast, 18 л</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Работа</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>м2</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D17" s="6" t="n"/>
@@ -2391,17 +2325,17 @@
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>eps100_wall_insulation_work_unit_price</t>
+          <t>primer_unit_price</t>
         </is>
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>eps_wall_insulation_work_m2</t>
+          <t>bitumen_primer_aquamast_18l_item</t>
         </is>
       </c>
       <c r="N17" s="6" t="inlineStr">
         <is>
-          <t>eps100_wall_insulation_work_unit_price</t>
+          <t>primer_unit_price</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr"/>
@@ -2409,7 +2343,7 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Пеноплэкс ГЕО 100 мм</t>
+          <t>Мастика гидроизоляционная AquaMast, 18 кг</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -2419,7 +2353,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>м3</t>
+          <t>шт</t>
         </is>
       </c>
       <c r="D18" s="6" t="n"/>
@@ -2448,17 +2382,17 @@
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
-          <t>eps100_unit_price</t>
+          <t>mastic_unit_price</t>
         </is>
       </c>
       <c r="M18" s="6" t="inlineStr">
         <is>
-          <t>eps_geo_100_m3</t>
+          <t>bitumen_mastic_aquamast_18kg_item</t>
         </is>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>eps100_unit_price</t>
+          <t>mastic_unit_price</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr"/>
@@ -2466,17 +2400,17 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Клей-пена для ЭППС</t>
+          <t>Утепление торца плиты ЭППС 100 мм, работа</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Работа</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>баллон</t>
+          <t>м2</t>
         </is>
       </c>
       <c r="D19" s="6" t="n"/>
@@ -2505,20 +2439,134 @@
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
+          <t>eps100_wall_insulation_work_unit_price</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="inlineStr">
+        <is>
+          <t>eps_wall_insulation_work_m2</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
+        <is>
+          <t>eps100_wall_insulation_work_unit_price</t>
+        </is>
+      </c>
+      <c r="O19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Пеноплэкс ГЕО 100 мм</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="inlineStr"/>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Заполнить цену из price registry/fallback/review.</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>waterproofing</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>eps100_unit_price</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="inlineStr">
+        <is>
+          <t>eps_geo_100_m3</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
+        <is>
+          <t>eps100_unit_price</t>
+        </is>
+      </c>
+      <c r="O20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Клей-пена для ЭППС</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>баллон</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="inlineStr"/>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>price_registry_with_fallback</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>Заполнить цену из price registry/fallback/review.</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>waterproofing</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
           <t>glue_foam_unit_price</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="M21" s="6" t="inlineStr">
         <is>
           <t>eps_foam_glue_can</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>glue_foam_unit_price</t>
         </is>
       </c>
-      <c r="O19" s="6" t="inlineStr"/>
+      <c r="O21" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2531,7 +2579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2760,6 +2808,448 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Будущие detail-шаблоны</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr"/>
+      <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr"/>
+      <c r="M5" s="4" t="inlineStr"/>
+      <c r="N5" s="4" t="inlineStr"/>
+      <c r="O5" s="4" t="inlineStr"/>
+      <c r="P5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Арматура</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr"/>
+      <c r="C6" s="4" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr"/>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr"/>
+      <c r="K6" s="4" t="inlineStr"/>
+      <c r="L6" s="4" t="inlineStr"/>
+      <c r="M6" s="4" t="inlineStr"/>
+      <c r="N6" s="4" t="inlineStr"/>
+      <c r="O6" s="4" t="inlineStr"/>
+      <c r="P6" s="4" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Арматура</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Марка / позиция арматуры</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Диаметр, мм</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м/п</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Итоговая длина, м/п</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>Для foundation/floor slabs/load-bearing/lintels: spec_length_m является первичной единицей, если PDF дает м/п.</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr"/>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>rebar_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Балки</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr"/>
+      <c r="C8" s="4" t="inlineStr"/>
+      <c r="D8" s="4" t="inlineStr"/>
+      <c r="E8" s="4" t="inlineStr"/>
+      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr"/>
+      <c r="K8" s="4" t="inlineStr"/>
+      <c r="L8" s="4" t="inlineStr"/>
+      <c r="M8" s="4" t="inlineStr"/>
+      <c r="N8" s="4" t="inlineStr"/>
+      <c r="O8" s="4" t="inlineStr"/>
+      <c r="P8" s="4" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Балка</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Балка / позиция</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Высота, м</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Ширина, м</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr"/>
+      <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr">
+        <is>
+          <t>Для плит перекрытия с балками: геометрия балки и/или строка спецификации Ж/Б балок.</t>
+        </is>
+      </c>
+      <c r="N9" s="7" t="inlineStr"/>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P9" s="7" t="inlineStr">
+        <is>
+          <t>beam_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Перемычки</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr"/>
+      <c r="C10" s="4" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr"/>
+      <c r="K10" s="4" t="inlineStr"/>
+      <c r="L10" s="4" t="inlineStr"/>
+      <c r="M10" s="4" t="inlineStr"/>
+      <c r="N10" s="4" t="inlineStr"/>
+      <c r="O10" s="4" t="inlineStr"/>
+      <c r="P10" s="4" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Перемычка</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Перемычка / U-блок</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>Итоговая длина, м</t>
+        </is>
+      </c>
+      <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>Для load_bearing_walls_lintels: длины перемычек и арматуры перемычек.</t>
+        </is>
+      </c>
+      <c r="N11" s="7" t="inlineStr"/>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P11" s="7" t="inlineStr">
+        <is>
+          <t>lintel_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Вентканалы / сегменты</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+      <c r="J12" s="4" t="inlineStr"/>
+      <c r="K12" s="4" t="inlineStr"/>
+      <c r="L12" s="4" t="inlineStr"/>
+      <c r="M12" s="4" t="inlineStr"/>
+      <c r="N12" s="4" t="inlineStr"/>
+      <c r="O12" s="4" t="inlineStr"/>
+      <c r="P12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Вентканал</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Сегмент / канал</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr">
+        <is>
+          <t>Для Schiedel и обкладки вентканалов, если PDF дает повторяющиеся сегменты.</t>
+        </is>
+      </c>
+      <c r="N13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P13" s="7" t="inlineStr">
+        <is>
+          <t>vent_chimney_cladding_segments</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Спецификация материалов</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr"/>
+      <c r="D14" s="4" t="inlineStr"/>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr"/>
+      <c r="K14" s="4" t="inlineStr"/>
+      <c r="L14" s="4" t="inlineStr"/>
+      <c r="M14" s="4" t="inlineStr"/>
+      <c r="N14" s="4" t="inlineStr"/>
+      <c r="O14" s="4" t="inlineStr"/>
+      <c r="P14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Материал / строка спецификации</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Объем, м3</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr"/>
+      <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr">
+        <is>
+          <t>Для ЭППС, бетона, опалубки, мембран и других строк спецификаций, которые не являются отдельной геометрией.</t>
+        </is>
+      </c>
+      <c r="N15" s="7" t="inlineStr"/>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P15" s="7" t="inlineStr">
+        <is>
+          <t>material_spec_rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Сырые строки таблиц</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr"/>
+      <c r="D16" s="4" t="inlineStr"/>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr"/>
+      <c r="K16" s="4" t="inlineStr"/>
+      <c r="L16" s="4" t="inlineStr"/>
+      <c r="M16" s="4" t="inlineStr"/>
+      <c r="N16" s="4" t="inlineStr"/>
+      <c r="O16" s="4" t="inlineStr"/>
+      <c r="P16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Raw row</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Сырая строка PDF</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr"/>
+      <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr">
+        <is>
+          <t>Raw table row from chat extraction before mapping to target_code.</t>
+        </is>
+      </c>
+      <c r="N17" s="7" t="inlineStr"/>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P17" s="7" t="inlineStr">
+        <is>
+          <t>raw_table_rows</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2861,136 +3351,677 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="100" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Блок 0: Summary запуска</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+      <c r="D1" s="8" t="n"/>
+      <c r="E1" s="8" t="n"/>
+      <c r="F1" s="8" t="n"/>
+      <c r="G1" s="8" t="n"/>
+      <c r="H1" s="8" t="n"/>
+      <c r="I1" s="8" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="n"/>
+      <c r="E2" s="9" t="n"/>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>section_contracts</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>workbook собран локально из section_contract.yaml</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="10" t="n"/>
+      <c r="I3" s="10" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>sections_count</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>сколько section contracts загружено</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="n"/>
+      <c r="E4" s="10" t="n"/>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
+      <c r="I4" s="10" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>review_parameters_count</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>сколько строк проверки проекта</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>price_rows_count</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>сколько строк цен</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>detail_templates_count</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>сколько detail-шаблонов</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>defaults_count</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>числовые default/ручные параметры остаются в contracts</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="10" t="n"/>
+      <c r="I8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>auto_calculated_count</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>поля, которые должны считаться кодом, а не извлекаться из PDF</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="10" t="n"/>
+      <c r="I9" s="10" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>parser_candidates_connected</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>будет заполнено на шаге extraction JSON -&gt; workbook</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n"/>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="10" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Блок 1: section contracts</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>section_code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B13" s="9" t="inlineStr">
         <is>
           <t>section_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D13" s="9" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E13" s="9" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G13" s="9" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>source_files</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C14" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="D2" s="8" t="n">
+      <c r="D14" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="E2" s="8" t="n">
+      <c r="E14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F14" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H14" s="10" t="n">
         <v>11</v>
       </c>
-      <c r="I2" s="8" t="inlineStr">
+      <c r="I14" s="10" t="inlineStr">
         <is>
           <t>{"calculator": "experiments/earthworks_calculator/earthworks_calculator.py", "calculator_readme": "experiments/earthworks_calculator/README.md", "existing_cases": [], "related_docs": ["experiments/full_estimate_review_pipeline/reports/step_01_earthworks_reference.md", "docs/report_earthworks_parser_google_stage1.md", "docs/report_earthworks_review_to_calculator.md"], "extraction_targets": ["experiments/chat_extraction_poc/data/calculator_targets_compact.json", "experiments/chat_extraction_poc/data/target_aliases_ru.yaml"]}</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C15" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D15" s="10" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E15" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F15" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G15" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H15" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>{"calculator": "experiments/waterproofing_calculator/waterproofing_calculator.py", "calculator_readme": "experiments/waterproofing_calculator/README.md", "existing_cases": ["experiments/waterproofing_calculator/cases/test_waterproofing_spec_area"], "related_docs": ["experiments/full_estimate_review_pipeline/reports/step_03_all_sections_quantity_matrix.md", "experiments/full_estimate_review_pipeline/reports/step_03b_production_contamination_audit.md", "docs/elena_parameter_review_pack_audit.md", "docs/report_paid_waterproofing_calculator_changes.md", "docs/report_waterproofing_calculator.md"], "extraction_targets": ["experiments/chat_extraction_poc/data/calculator_targets_compact.json", "experiments/chat_extraction_poc/data/target_aliases_ru.yaml"]}</t>
         </is>
       </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Блок 2: planned detail groups</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>detail_table_key</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>used_for</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>trench_routes</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Маршруты траншей</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>детальная таблица уже описана в section_contract.yaml</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="10" t="n"/>
+      <c r="I19" s="10" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>communications_pipe_items</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>Трубы коммуникаций</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>contract</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>earthworks</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>детальная таблица уже описана в section_contract.yaml</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="10" t="n"/>
+      <c r="H20" s="10" t="n"/>
+      <c r="I20" s="10" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>rebar_items</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>Арматура</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Арматура</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>future sections</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Для foundation/floor slabs/load-bearing/lintels: spec_length_m является первичной единицей, если PDF дает м/п.</t>
+        </is>
+      </c>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="10" t="n"/>
+      <c r="I21" s="10" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>beam_items</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Балки</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Балка</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t>future sections</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="inlineStr">
+        <is>
+          <t>Для плит перекрытия с балками: геометрия балки и/или строка спецификации Ж/Б балок.</t>
+        </is>
+      </c>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>lintel_items</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Перемычки</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Перемычка</t>
+        </is>
+      </c>
+      <c r="D23" s="10" t="inlineStr">
+        <is>
+          <t>future sections</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="inlineStr">
+        <is>
+          <t>Для load_bearing_walls_lintels: длины перемычек и арматуры перемычек.</t>
+        </is>
+      </c>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
+      <c r="H23" s="10" t="n"/>
+      <c r="I23" s="10" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>vent_chimney_cladding_segments</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>Вентканалы / сегменты</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Вентканал</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>future sections</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>Для Schiedel и обкладки вентканалов, если PDF дает повторяющиеся сегменты.</t>
+        </is>
+      </c>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="10" t="n"/>
+      <c r="I24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>material_spec_rows</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>Спецификация материалов</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>future sections</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>Для ЭППС, бетона, опалубки, мембран и других строк спецификаций, которые не являются отдельной геометрией.</t>
+        </is>
+      </c>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="10" t="n"/>
+      <c r="I25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>raw_table_rows</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Сырые строки таблиц</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>Raw row</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>future sections</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>Raw table row from chat extraction before mapping to target_code.</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="10" t="n"/>
+      <c r="I26" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3003,7 +4034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3012,34 +4043,123 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Блок 0: Summary запуска</t>
+        </is>
+      </c>
+      <c r="B1" s="8" t="n"/>
+      <c r="C1" s="8" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Комментарий</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>section_contracts</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>сырые parser/chat данные подключаются следующим шагом</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>sections_count</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>сколько section contracts загружено</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>raw_parser_json_connected</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>пока лист показывает сырье contracts для диагностики</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Блок 1: raw contract blocks</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n"/>
+      <c r="C7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>section_code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>block</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>json</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>{
   "code": "earthworks",
@@ -3051,18 +4171,18 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -3311,18 +4431,18 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -3485,18 +4605,18 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -3632,18 +4752,18 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -3771,18 +4891,18 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -3825,18 +4945,18 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -4176,18 +5296,18 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>{
   "code": "waterproofing",
@@ -4199,18 +5319,18 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -4289,18 +5409,18 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -4385,35 +5505,35 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C20" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -4574,18 +5694,18 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C21" s="10" t="inlineStr">
         <is>
           <t>[
   {
@@ -4738,18 +5858,18 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C22" s="10" t="inlineStr">
         <is>
           <t>[
   {

</xml_diff>

<commit_message>
Match review workbook earthworks detail styling
</commit_message>
<xml_diff>
--- a/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
+++ b/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
@@ -43,7 +43,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00000000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -52,7 +52,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -66,7 +66,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00666666"/>
+        <fgColor rgb="00E7E6E6"/>
       </patternFill>
     </fill>
     <fill>
@@ -81,12 +81,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DAE8FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -139,13 +134,13 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2579,7 +2574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2809,31 +2804,27 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Будущие detail-шаблоны</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr"/>
-      <c r="C5" s="4" t="inlineStr"/>
-      <c r="D5" s="4" t="inlineStr"/>
-      <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="4" t="inlineStr"/>
-      <c r="G5" s="4" t="inlineStr"/>
-      <c r="H5" s="4" t="inlineStr"/>
-      <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" s="4" t="inlineStr"/>
-      <c r="K5" s="4" t="inlineStr"/>
-      <c r="L5" s="4" t="inlineStr"/>
-      <c r="M5" s="4" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="4" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr"/>
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="n"/>
+      <c r="O5" s="2" t="n"/>
+      <c r="P5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Арматура</t>
+          <t>Будущие detail-шаблоны</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr"/>
@@ -2853,63 +2844,27 @@
       <c r="P6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Арматура</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Марка / позиция арматуры</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Диаметр, мм</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Длина, м/п</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>Количество</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>Итоговая длина, м/п</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>Для foundation/floor slabs/load-bearing/lintels: spec_length_m является первичной единицей, если PDF дает м/п.</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr"/>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-      <c r="P7" s="7" t="inlineStr">
-        <is>
-          <t>rebar_items</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="n"/>
+      <c r="O7" s="2" t="n"/>
+      <c r="P7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Балки</t>
+          <t>Арматура</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr"/>
@@ -2931,43 +2886,43 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Балка</t>
+          <t>Арматура</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Балка / позиция</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Длина, м</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Высота, м</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Ширина, м</t>
-        </is>
-      </c>
+          <t>Марка / позиция арматуры</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
       <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>Диаметр, мм</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м/п</t>
+        </is>
+      </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
           <t>Количество</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>Итоговая длина, м/п</t>
+        </is>
+      </c>
       <c r="K9" s="7" t="inlineStr"/>
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Для плит перекрытия с балками: геометрия балки и/или строка спецификации Ж/Б балок.</t>
+          <t>Для foundation/floor slabs/load-bearing/lintels: spec_length_m является первичной единицей, если PDF дает м/п.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr"/>
@@ -2978,154 +2933,126 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
+          <t>rebar_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Балки</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr"/>
+      <c r="C11" s="4" t="inlineStr"/>
+      <c r="D11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr"/>
+      <c r="K11" s="4" t="inlineStr"/>
+      <c r="L11" s="4" t="inlineStr"/>
+      <c r="M11" s="4" t="inlineStr"/>
+      <c r="N11" s="4" t="inlineStr"/>
+      <c r="O11" s="4" t="inlineStr"/>
+      <c r="P11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Балка</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Балка / позиция</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Высота, м</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Ширина, м</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="inlineStr"/>
+      <c r="K12" s="7" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
+      <c r="M12" s="7" t="inlineStr">
+        <is>
+          <t>Для плит перекрытия с балками: геометрия балки и/или строка спецификации Ж/Б балок.</t>
+        </is>
+      </c>
+      <c r="N12" s="7" t="inlineStr"/>
+      <c r="O12" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P12" s="7" t="inlineStr">
+        <is>
           <t>beam_items</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Перемычки</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="4" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="4" t="inlineStr"/>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr"/>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="4" t="inlineStr"/>
-      <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr"/>
-      <c r="O10" s="4" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>Перемычка</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Перемычка / U-блок</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Длина, м</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>Количество</t>
-        </is>
-      </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>Итоговая длина, м</t>
-        </is>
-      </c>
-      <c r="K11" s="7" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>Для load_bearing_walls_lintels: длины перемычек и арматуры перемычек.</t>
-        </is>
-      </c>
-      <c r="N11" s="7" t="inlineStr"/>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-      <c r="P11" s="7" t="inlineStr">
-        <is>
-          <t>lintel_items</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Вентканалы / сегменты</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr"/>
-      <c r="C12" s="4" t="inlineStr"/>
-      <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="4" t="inlineStr"/>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr"/>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="4" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>Вентканал</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Сегмент / канал</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>Длина, м</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>Количество</t>
-        </is>
-      </c>
-      <c r="J13" s="7" t="inlineStr"/>
-      <c r="K13" s="7" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
-      <c r="M13" s="7" t="inlineStr">
-        <is>
-          <t>Для Schiedel и обкладки вентканалов, если PDF дает повторяющиеся сегменты.</t>
-        </is>
-      </c>
-      <c r="N13" s="7" t="inlineStr"/>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>template</t>
-        </is>
-      </c>
-      <c r="P13" s="7" t="inlineStr">
-        <is>
-          <t>vent_chimney_cladding_segments</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Спецификация материалов</t>
+          <t>Перемычки</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr"/>
@@ -3147,22 +3074,22 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Материал</t>
+          <t>Перемычка</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Материал / строка спецификации</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr"/>
+          <t>Перемычка / U-блок</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м</t>
+        </is>
+      </c>
       <c r="D15" s="7" t="inlineStr"/>
       <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Объем, м3</t>
-        </is>
-      </c>
+      <c r="F15" s="7" t="inlineStr"/>
       <c r="G15" s="7" t="inlineStr"/>
       <c r="H15" s="7" t="inlineStr"/>
       <c r="I15" s="7" t="inlineStr">
@@ -3170,12 +3097,16 @@
           <t>Количество</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>Итоговая длина, м</t>
+        </is>
+      </c>
       <c r="K15" s="7" t="inlineStr"/>
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Для ЭППС, бетона, опалубки, мембран и других строк спецификаций, которые не являются отдельной геометрией.</t>
+          <t>Для load_bearing_walls_lintels: длины перемычек и арматуры перемычек.</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr"/>
@@ -3186,65 +3117,255 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
+          <t>lintel_items</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="n"/>
+      <c r="O16" s="2" t="n"/>
+      <c r="P16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Вентканалы / сегменты</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr"/>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="inlineStr"/>
+      <c r="E17" s="4" t="inlineStr"/>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
+      <c r="K17" s="4" t="inlineStr"/>
+      <c r="L17" s="4" t="inlineStr"/>
+      <c r="M17" s="4" t="inlineStr"/>
+      <c r="N17" s="4" t="inlineStr"/>
+      <c r="O17" s="4" t="inlineStr"/>
+      <c r="P17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Вентканал</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Сегмент / канал</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Длина, м</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr"/>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="inlineStr"/>
+      <c r="K18" s="7" t="inlineStr"/>
+      <c r="L18" s="7" t="inlineStr"/>
+      <c r="M18" s="7" t="inlineStr">
+        <is>
+          <t>Для Schiedel и обкладки вентканалов, если PDF дает повторяющиеся сегменты.</t>
+        </is>
+      </c>
+      <c r="N18" s="7" t="inlineStr"/>
+      <c r="O18" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P18" s="7" t="inlineStr">
+        <is>
+          <t>vent_chimney_cladding_segments</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="n"/>
+      <c r="P19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Спецификация материалов</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr"/>
+      <c r="C20" s="4" t="inlineStr"/>
+      <c r="D20" s="4" t="inlineStr"/>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr"/>
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
+      <c r="J20" s="4" t="inlineStr"/>
+      <c r="K20" s="4" t="inlineStr"/>
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="4" t="inlineStr"/>
+      <c r="N20" s="4" t="inlineStr"/>
+      <c r="O20" s="4" t="inlineStr"/>
+      <c r="P20" s="4" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Материал</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Материал / строка спецификации</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr"/>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Объем, м3</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>Количество</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr"/>
+      <c r="K21" s="7" t="inlineStr"/>
+      <c r="L21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>Для ЭППС, бетона, опалубки, мембран и других строк спецификаций, которые не являются отдельной геометрией.</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr"/>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>template</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
           <t>material_spec_rows</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="n"/>
+      <c r="P22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Сырые строки таблиц</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr"/>
-      <c r="C16" s="4" t="inlineStr"/>
-      <c r="D16" s="4" t="inlineStr"/>
-      <c r="E16" s="4" t="inlineStr"/>
-      <c r="F16" s="4" t="inlineStr"/>
-      <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr"/>
-      <c r="I16" s="4" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr"/>
-      <c r="K16" s="4" t="inlineStr"/>
-      <c r="L16" s="4" t="inlineStr"/>
-      <c r="M16" s="4" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="4" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr"/>
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
+      <c r="K23" s="4" t="inlineStr"/>
+      <c r="L23" s="4" t="inlineStr"/>
+      <c r="M23" s="4" t="inlineStr"/>
+      <c r="N23" s="4" t="inlineStr"/>
+      <c r="O23" s="4" t="inlineStr"/>
+      <c r="P23" s="4" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>Raw row</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Сырая строка PDF</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr"/>
-      <c r="D17" s="7" t="inlineStr"/>
-      <c r="E17" s="7" t="inlineStr"/>
-      <c r="F17" s="7" t="inlineStr"/>
-      <c r="G17" s="7" t="inlineStr"/>
-      <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr"/>
-      <c r="J17" s="7" t="inlineStr"/>
-      <c r="K17" s="7" t="inlineStr"/>
-      <c r="L17" s="7" t="inlineStr"/>
-      <c r="M17" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr"/>
+      <c r="E24" s="7" t="inlineStr"/>
+      <c r="F24" s="7" t="inlineStr"/>
+      <c r="G24" s="7" t="inlineStr"/>
+      <c r="H24" s="7" t="inlineStr"/>
+      <c r="I24" s="7" t="inlineStr"/>
+      <c r="J24" s="7" t="inlineStr"/>
+      <c r="K24" s="7" t="inlineStr"/>
+      <c r="L24" s="7" t="inlineStr"/>
+      <c r="M24" s="7" t="inlineStr">
         <is>
           <t>Raw table row from chat extraction before mapping to target_code.</t>
         </is>
       </c>
-      <c r="N17" s="7" t="inlineStr"/>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="N24" s="7" t="inlineStr"/>
+      <c r="O24" s="7" t="inlineStr">
         <is>
           <t>template</t>
         </is>
       </c>
-      <c r="P17" s="7" t="inlineStr">
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>raw_table_rows</t>
         </is>

</xml_diff>

<commit_message>
Use white background for parser technical sheets
</commit_message>
<xml_diff>
--- a/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
+++ b/experiments/full_estimate_review_pipeline/output/step_06_earthworks_waterproofing_review.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -139,9 +139,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3525,187 +3522,187 @@
       <c r="I2" s="9" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>section_contracts</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>workbook собран локально из section_contract.yaml</t>
         </is>
       </c>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>sections_count</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>сколько section contracts загружено</t>
         </is>
       </c>
-      <c r="D4" s="10" t="n"/>
-      <c r="E4" s="10" t="n"/>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
-      <c r="I4" s="10" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>review_parameters_count</t>
         </is>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>сколько строк проверки проекта</t>
         </is>
       </c>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>price_rows_count</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="7" t="n">
         <v>18</v>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>сколько строк цен</t>
         </is>
       </c>
-      <c r="D6" s="10" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>detail_templates_count</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>сколько detail-шаблонов</t>
         </is>
       </c>
-      <c r="D7" s="10" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>defaults_count</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="7" t="n">
         <v>25</v>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>числовые default/ручные параметры остаются в contracts</t>
         </is>
       </c>
-      <c r="D8" s="10" t="n"/>
-      <c r="E8" s="10" t="n"/>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="7" t="n"/>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>auto_calculated_count</t>
         </is>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>поля, которые должны считаться кодом, а не извлекаться из PDF</t>
         </is>
       </c>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>parser_candidates_connected</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>будет заполнено на шаге extraction JSON -&gt; workbook</t>
         </is>
       </c>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="10" t="n"/>
-      <c r="E11" s="10" t="n"/>
-      <c r="F11" s="10" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
-      <c r="I11" s="10" t="n"/>
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="7" t="n"/>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -3770,85 +3767,85 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Земляные работы</t>
         </is>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="10" t="n">
+      <c r="F14" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="G14" s="10" t="n">
+      <c r="G14" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="10" t="n">
+      <c r="H14" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="I14" s="10" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>{"calculator": "experiments/earthworks_calculator/earthworks_calculator.py", "calculator_readme": "experiments/earthworks_calculator/README.md", "existing_cases": [], "related_docs": ["experiments/full_estimate_review_pipeline/reports/step_01_earthworks_reference.md", "docs/report_earthworks_parser_google_stage1.md", "docs/report_earthworks_review_to_calculator.md"], "extraction_targets": ["experiments/chat_extraction_poc/data/calculator_targets_compact.json", "experiments/chat_extraction_poc/data/target_aliases_ru.yaml"]}</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Гидроизоляция фундаментной плиты</t>
         </is>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="10" t="n">
+      <c r="F15" s="7" t="n">
         <v>14</v>
       </c>
-      <c r="G15" s="10" t="n">
+      <c r="G15" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="H15" s="10" t="n">
+      <c r="H15" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="I15" s="10" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>{"calculator": "experiments/waterproofing_calculator/waterproofing_calculator.py", "calculator_readme": "experiments/waterproofing_calculator/README.md", "existing_cases": ["experiments/waterproofing_calculator/cases/test_waterproofing_spec_area"], "related_docs": ["experiments/full_estimate_review_pipeline/reports/step_03_all_sections_quantity_matrix.md", "experiments/full_estimate_review_pipeline/reports/step_03b_production_contamination_audit.md", "docs/elena_parameter_review_pack_audit.md", "docs/report_paid_waterproofing_calculator_changes.md", "docs/report_waterproofing_calculator.md"], "extraction_targets": ["experiments/chat_extraction_poc/data/calculator_targets_compact.json", "experiments/chat_extraction_poc/data/target_aliases_ru.yaml"]}</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="n"/>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="10" t="n"/>
+      <c r="A16" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -3897,252 +3894,252 @@
       <c r="I18" s="9" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>trench_routes</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Маршруты траншей</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>contract</t>
         </is>
       </c>
-      <c r="D19" s="10" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>детальная таблица уже описана в section_contract.yaml</t>
         </is>
       </c>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="10" t="n"/>
-      <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>communications_pipe_items</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Трубы коммуникаций</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>contract</t>
         </is>
       </c>
-      <c r="D20" s="10" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>детальная таблица уже описана в section_contract.yaml</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="10" t="n"/>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>rebar_items</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Арматура</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Арматура</t>
         </is>
       </c>
-      <c r="D21" s="10" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>future sections</t>
         </is>
       </c>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>Для foundation/floor slabs/load-bearing/lintels: spec_length_m является первичной единицей, если PDF дает м/п.</t>
         </is>
       </c>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="10" t="n"/>
-      <c r="I21" s="10" t="n"/>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>beam_items</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Балки</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Балка</t>
         </is>
       </c>
-      <c r="D22" s="10" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>future sections</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Для плит перекрытия с балками: геометрия балки и/или строка спецификации Ж/Б балок.</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n"/>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>lintel_items</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Перемычки</t>
         </is>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Перемычка</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>future sections</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Для load_bearing_walls_lintels: длины перемычек и арматуры перемычек.</t>
         </is>
       </c>
-      <c r="F23" s="10" t="n"/>
-      <c r="G23" s="10" t="n"/>
-      <c r="H23" s="10" t="n"/>
-      <c r="I23" s="10" t="n"/>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>vent_chimney_cladding_segments</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Вентканалы / сегменты</t>
         </is>
       </c>
-      <c r="C24" s="10" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>Вентканал</t>
         </is>
       </c>
-      <c r="D24" s="10" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>future sections</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>Для Schiedel и обкладки вентканалов, если PDF дает повторяющиеся сегменты.</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="10" t="n"/>
-      <c r="I24" s="10" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>material_spec_rows</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Спецификация материалов</t>
         </is>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Материал</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>future sections</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>Для ЭППС, бетона, опалубки, мембран и других строк спецификаций, которые не являются отдельной геометрией.</t>
         </is>
       </c>
-      <c r="F25" s="10" t="n"/>
-      <c r="G25" s="10" t="n"/>
-      <c r="H25" s="10" t="n"/>
-      <c r="I25" s="10" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>raw_table_rows</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Сырые строки таблиц</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>Raw row</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>future sections</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="7" t="inlineStr">
         <is>
           <t>Raw table row from chat extraction before mapping to target_code.</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="10" t="n"/>
-      <c r="I26" s="10" t="n"/>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4190,58 +4187,58 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>section_contracts</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>сырые parser/chat данные подключаются следующим шагом</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>sections_count</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>сколько section contracts загружено</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>raw_parser_json_connected</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>нет</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>пока лист показывает сырье contracts для диагностики</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n"/>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10" t="n"/>
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -4270,17 +4267,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>{
   "code": "earthworks",
@@ -4293,17 +4290,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="C10" s="10" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -4553,17 +4550,17 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -4727,17 +4724,17 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -4874,17 +4871,17 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5013,17 +5010,17 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5067,17 +5064,17 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>earthworks</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5418,17 +5415,17 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>{
   "code": "waterproofing",
@@ -5441,17 +5438,17 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>review_parameters</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5531,17 +5528,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>price_keys</t>
         </is>
       </c>
-      <c r="C18" s="10" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5627,34 +5624,34 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>detail_tables</t>
         </is>
       </c>
-      <c r="C19" s="10" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>defaults</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5816,17 +5813,17 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>auto_calculated</t>
         </is>
       </c>
-      <c r="C21" s="10" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>[
   {
@@ -5980,17 +5977,17 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>waterproofing</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>estimate_lines</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>[
   {

</xml_diff>